<commit_message>
fix: clarify template namespaces and rendering
Clarify implemented template namespaces and rendering behavior in docs, and align resolver/tests/examples with the supported namespaces.

Fixes #7
</commit_message>
<xml_diff>
--- a/examples/product_analysis.xlsx
+++ b/examples/product_analysis.xlsx
@@ -419,103 +419,103 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>avg_profit_per_unit</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_profit</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>total_revenue</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>total_units</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>product</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>total_revenue</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>total_profit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>avg_profit_per_unit</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>675</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Widget A</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Widget C</t>
+          <t>14.99</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>13493.25</t>
+          <t>7794.80</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8093.25</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>11.99</t>
-        </is>
+          <t>15594.80</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>520</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Widget B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>24.99</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>7172.13</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>14347.13</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
         <v>287</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Widget B</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>14347.13</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>7172.13</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>24.99</t>
-        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>520</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Widget C</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Widget A</t>
+          <t>11.99</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>15594.80</t>
+          <t>8093.25</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>7794.80</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>14.99</t>
-        </is>
+          <t>13493.25</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>